<commit_message>
adding analysis for G1
</commit_message>
<xml_diff>
--- a/dataset_t6_grouped/results2/G0/G0_DMSO_W0082F0001T0006Z000C1N11_analysis.xlsx
+++ b/dataset_t6_grouped/results2/G0/G0_DMSO_W0082F0001T0006Z000C1N11_analysis.xlsx
@@ -480,16 +480,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>41.15660033262248</v>
+        <v>6.687947554051154</v>
       </c>
       <c r="D2" t="n">
-        <v>40.9637423380314</v>
+        <v>6.656608129930103</v>
       </c>
       <c r="E2" t="n">
-        <v>5.769841129392417</v>
+        <v>0.9375991835262679</v>
       </c>
       <c r="F2" t="n">
-        <v>5.664928781655258</v>
+        <v>0.9205509270189794</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -512,16 +512,16 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>42.85633705318391</v>
+        <v>6.964154771142385</v>
       </c>
       <c r="D3" t="n">
-        <v>42.09488258180621</v>
+        <v>6.84041841954351</v>
       </c>
       <c r="E3" t="n">
-        <v>5.769841129392417</v>
+        <v>0.9375991835262679</v>
       </c>
       <c r="F3" t="n">
-        <v>5.664928781655258</v>
+        <v>0.9205509270189794</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -544,16 +544,16 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>34.1139522753398</v>
+        <v>5.543517244742717</v>
       </c>
       <c r="D4" t="n">
-        <v>33.22275787731303</v>
+        <v>5.398698155063367</v>
       </c>
       <c r="E4" t="n">
-        <v>5.769841129392417</v>
+        <v>0.9375991835262679</v>
       </c>
       <c r="F4" t="n">
-        <v>5.664928781655258</v>
+        <v>0.9205509270189794</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -576,16 +576,16 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>35.89303540006349</v>
+        <v>5.832618252510318</v>
       </c>
       <c r="D5" t="n">
-        <v>35.09020504548374</v>
+        <v>5.702158319891108</v>
       </c>
       <c r="E5" t="n">
-        <v>5.769841129392417</v>
+        <v>0.9375991835262679</v>
       </c>
       <c r="F5" t="n">
-        <v>5.664928781655258</v>
+        <v>0.9205509270189794</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -608,16 +608,16 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>44.18782139798616</v>
+        <v>7.180520977172752</v>
       </c>
       <c r="D6" t="n">
-        <v>43.41245863544228</v>
+        <v>7.054524528259371</v>
       </c>
       <c r="E6" t="n">
-        <v>5.769841129392417</v>
+        <v>0.9375991835262679</v>
       </c>
       <c r="F6" t="n">
-        <v>5.664928781655258</v>
+        <v>0.9205509270189794</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -640,16 +640,16 @@
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>25.34227138469009</v>
+        <v>4.118119100012139</v>
       </c>
       <c r="D7" t="n">
-        <v>25.22134605482525</v>
+        <v>4.098468733909104</v>
       </c>
       <c r="E7" t="n">
-        <v>5.769841129392417</v>
+        <v>0.9375991835262679</v>
       </c>
       <c r="F7" t="n">
-        <v>5.664928781655258</v>
+        <v>0.9205509270189794</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -672,16 +672,16 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>34.92429505721174</v>
+        <v>5.675197946796908</v>
       </c>
       <c r="D8" t="n">
-        <v>35.17162400353879</v>
+        <v>5.715388900575054</v>
       </c>
       <c r="E8" t="n">
-        <v>5.769841129392417</v>
+        <v>0.9375991835262679</v>
       </c>
       <c r="F8" t="n">
-        <v>5.664928781655258</v>
+        <v>0.9205509270189794</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -704,16 +704,16 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>40.83290028905047</v>
+        <v>6.635346296970702</v>
       </c>
       <c r="D9" t="n">
-        <v>40.73484749903839</v>
+        <v>6.619412718593738</v>
       </c>
       <c r="E9" t="n">
-        <v>5.769841129392417</v>
+        <v>0.9375991835262679</v>
       </c>
       <c r="F9" t="n">
-        <v>5.664928781655258</v>
+        <v>0.9205509270189794</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>

</xml_diff>